<commit_message>
AASPCNJ01: sobrenomes (Raony Chagas/Levi Santos) + guia de evidências
- Aplica sobrenomes nos 18 .md e na planilha; regenera os 18 .docx.
- Índice -> v1.4.
- Cria _interno/COLETA-EVIDENCIAS_AASPCNJ_Tech-Lead (.md + .docx):
  guia por documento/processo do que o Raony deve levantar (prints,
  exports e links de Azure DevOps, ClickUp, RabbitMQ, banco, Elastic,
  Postman) para sustentar as referências técnicas dos registros.

https://claude.ai/code/session_01Lvzca1A5yJyk8RTZH29onh
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_CNJ/GEST-AASPCNJ01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_CNJ/GEST-AASPCNJ01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -95,7 +95,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -117,11 +117,55 @@
         <color rgb="00BBBBBB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -169,6 +213,8 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -559,6 +605,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -577,6 +624,8 @@
           <t>AASP — Associação dos Advogados de São Paulo</t>
         </is>
       </c>
+      <c r="C5" s="19" t="n"/>
+      <c r="D5" s="20" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -589,6 +638,8 @@
           <t>WorkerAndamentos — Agente de Captura de Andamentos Processuais (.NET)</t>
         </is>
       </c>
+      <c r="C6" s="19" t="n"/>
+      <c r="D6" s="20" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -601,6 +652,8 @@
           <t>AASPCNJ01</t>
         </is>
       </c>
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="20" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -613,6 +666,8 @@
           <t>Abraão Oliveira</t>
         </is>
       </c>
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="20" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -625,6 +680,8 @@
           <t>Cézar</t>
         </is>
       </c>
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="20" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -634,9 +691,11 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Raony</t>
-        </is>
-      </c>
+          <t>Raony Chagas</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="20" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -646,9 +705,11 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Levi (desde abr/2026)</t>
-        </is>
-      </c>
+          <t>Levi Santos (desde abr/2026)</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="20" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -661,6 +722,8 @@
           <t>Jonatan (desde a Fase 5)</t>
         </is>
       </c>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="20" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -673,6 +736,8 @@
           <t>David</t>
         </is>
       </c>
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="20" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -685,6 +750,8 @@
           <t>Carlos Alves</t>
         </is>
       </c>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="20" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -697,6 +764,8 @@
           <t>Wilson Yamada</t>
         </is>
       </c>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="20" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -709,6 +778,8 @@
           <t>01/10/2025</t>
         </is>
       </c>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="20" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -721,6 +792,8 @@
           <t>30/06/2026</t>
         </is>
       </c>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="20" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -733,7 +806,10 @@
           <t>Em execução — desenvolvimento concluído; implantação (Fase 6) em andamento</t>
         </is>
       </c>
-    </row>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="20" t="n"/>
+    </row>
+    <row r="19"/>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -1188,6 +1264,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1199,6 +1276,8 @@
           <t>Wilson Yamada</t>
         </is>
       </c>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="20" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1211,6 +1290,8 @@
           <t>Sim — não participa da execução do projeto</t>
         </is>
       </c>
+      <c r="C5" s="19" t="n"/>
+      <c r="D5" s="20" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1223,6 +1304,8 @@
           <t>Desenvolvimento / Homologação (execução)</t>
         </is>
       </c>
+      <c r="C6" s="19" t="n"/>
+      <c r="D6" s="20" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1235,6 +1318,8 @@
           <t>11/06/2026</t>
         </is>
       </c>
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="20" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1247,6 +1332,8 @@
           <t>Conforme com ressalvas</t>
         </is>
       </c>
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="20" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1259,7 +1346,10 @@
           <t>88,9% (8/9 itens de processo)</t>
         </is>
       </c>
-    </row>
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="20" t="n"/>
+    </row>
+    <row r="10"/>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -1529,6 +1619,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
@@ -1666,6 +1757,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1895,6 +1987,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -2192,6 +2285,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
@@ -2442,6 +2536,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2705,6 +2800,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -3203,6 +3299,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3506,6 +3603,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -4296,7 +4394,7 @@
           <t>TOTAL — 20 histórias</t>
         </is>
       </c>
-      <c r="B36" s="14" t="n"/>
+      <c r="B36" s="20" t="n"/>
       <c r="C36" s="14" t="n"/>
       <c r="D36" s="15" t="inlineStr">
         <is>
@@ -4351,6 +4449,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -6210,6 +6309,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -6301,7 +6401,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Raony</t>
+          <t>Raony Chagas</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -6328,7 +6428,7 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Levi</t>
+          <t>Levi Santos</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -6433,6 +6533,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -6565,6 +6666,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -7160,6 +7262,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -7392,6 +7495,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -7763,6 +7867,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -7847,6 +7952,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -7949,6 +8055,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -8333,6 +8440,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
AASPCNJ01: confirma sobrenome do Arquiteto (Cézar Hiraki)
Aplica "Cézar Hiraki" nos 18 .md e na planilha; regenera os 18 .docx.
Índice -> v1.5; equipe completa. Mesma pessoa do projeto FTGASMIG.

https://claude.ai/code/session_01Lvzca1A5yJyk8RTZH29onh
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_CNJ/GEST-AASPCNJ01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_CNJ/GEST-AASPCNJ01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -677,7 +677,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Cézar</t>
+          <t>Cézar Hiraki</t>
         </is>
       </c>
       <c r="C9" s="19" t="n"/>
@@ -6374,7 +6374,7 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Cézar</t>
+          <t>Cézar Hiraki</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">

</xml_diff>

<commit_message>
docs(CNJ): recria modelagem ágil na GEST (Discovery + 11 sprints, 155 SP, épicos/US) e remove contradição de SP no ADAP
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_CNJ/GEST-AASPCNJ01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_CNJ/GEST-AASPCNJ01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -18,6 +18,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medição" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GQA" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V&amp;V — Testes" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog Ágil (Jira)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprints e Velocity" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -2154,7 +2156,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="21.75" customHeight="1" s="59">
       <c r="A22" s="62" t="inlineStr">
         <is>
@@ -2648,7 +2649,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="21.75" customHeight="1" s="59">
       <c r="A12" s="62" t="inlineStr">
         <is>
@@ -2739,6 +2739,1931 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" style="59" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>BACKLOG DO PROJETO — ÉPICOS E HISTÓRIAS (base Jira)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Derivado de REQ-AASPCNJ01-001 · Tipo: Epic / Story · Pronto para carga no Jira</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ÉPICOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Resumo</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>RF/RNF</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EP-01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Captura EPROC/ESAJ (TJSP)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>RF-02</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Disc.–S5</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EP-02</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Integração DataJud/CNJ (fonte primária)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>RF-01,05,06,11</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>S2,S6,S7,S8</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EP-03</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fila unificada (RabbitMQ)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>RF-03,12</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>S2,S6</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EP-04</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Fallback e APIs parceiras</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>RF-04,07,08</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>S7,S8</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Segredo de justiça por instância</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>RF-10</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Observabilidade e estabilidade</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>RF-09,RNF-02,03</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>S7,S8</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>EP-07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Qualidade, testes e implantação</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>RNF / VV</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>S10,S11</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HISTÓRIAS DE USUÁRIO (User Stories)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>História</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>RF/RNF</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Épico</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>US-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Como operação, quero capturar processos do TJSP via engine EPROC/ESAJ para não depender de APIs privadas no maior tribunal</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>RF-02</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>EP-01</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>US-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Como operação, quero contornar o captcha Cloudflare nos portais do TJSP para viabilizar a captura automatizada</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>RF-02</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>EP-01</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>US-03</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Como operação, quero capturar a 1ª instância (EPROC) e os incidentes (ESAJ) do TJSP</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>RF-02</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>EP-01</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>US-19</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Como operação, quero estabilizar o crawler EPROC (timeout pós-captcha, nullabilidade) para captura confiável</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>RNF-02</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>EP-01</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>US-20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Como operação, quero melhorar o desempenho do crawler e preparar o pacote de GMUD do EPROC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>RNF-01</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>EP-01</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>US-04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Como operação, quero consultar a API DataJud/CNJ como fonte primária para NUPs com CodigoFonteAPI nulo</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>RF-01</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>EP-02</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>US-06</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Como sistema, quero registrar o CodigoFonteAPI por processo para rastrear a fonte de cada captura</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>RF-06</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>EP-02</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>US-07</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Como sistema, quero enviar os dados capturados ao webhook da API AndamentosProcessuais para indexação no Elasticsearch</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>RF-11</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>EP-02</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>US-05</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Como sistema, quero gerenciar o token Bearer da CNJ de forma compartilhada com renovação automática</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>RF-05</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>EP-02</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>US-08</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Como sistema, quero que o CapturaServer enfileire todos os NUPs no RabbitMQ de forma unificada</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>RF-12</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>EP-03</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>US-09</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Como worker, quero ler a fila unificada independente do tribunal de origem</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>RF-03</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>EP-03</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>US-10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Como sistema, quero desligar o NUP nas APIs parceiras após captura via CNJ, registrando log</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>RF-04</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>EP-04</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>US-11</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Como sistema, quero fazer fallback para as parceiras por ordem de prioridade quando CNJ e EPROC falham</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>RF-07</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>EP-04</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>US-12</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Como sistema, quero tratar todos os retornos das parceiras (NUP inválido, vazio/aguardando, erro total e parcial)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>RF-08</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>EP-04</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>US-13</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Como operação, quero controlar o segredo de justiça por instância (campo Segredo) sem impactar instâncias não restritas</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>RF-10</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>EP-05</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>US-14</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Como operação, quero registrar erros detalhados por instância nas tabelas de controle</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>RF-09</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>US-15</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Como operação, quero que a fila se recupere de travamentos sem intervenção manual (incidente de 137 mil itens)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>RNF-02</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>EP-06</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>US-16</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Como QA, quero validar o fluxo completo (sucesso, fallback e erro parcial) por amostragem (E2E)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>VV</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>EP-07</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>US-17</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Como sistema, quero retry no envio ao webhook para aumentar a resiliência da entrega ao Elasticsearch</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>RNF-02</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>EP-07</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>US-18</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Como operação, quero implantar via GMUD e retomar a captura de 2ª instância no EPROC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Fase 6</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>EP-07</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>🟡 Em and.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TOTAL — 20 histórias</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" style="59" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ACOMPANHAMENTO DE SPRINTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Referência: RAC-AASPCNJ01-001 · MED-AASPCNJ01-001 · SP = modelagem retroativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EVOLUÇÃO POR SPRINT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Período</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SP Plan.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SP Real.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Desvio</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Velocity</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Defeitos</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Observação / eventos</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Out/25–09/01/26</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Estudo do captcha; arquitetura EPROC/ESAJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>12–23/01/26</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Crawler EPROC TJSP; webhook indexação</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>26/01–06/02/26</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Enfileiramento EprocTjsp; endpoint RabbitMQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09–20/02/26</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Proxy; 1ª instância; testes de desempenho</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>23/02–06/03/26</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Correções: navegador, timeout, nullabilidade (BUG-01..04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09–20/03/26</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Desempenho crawler; ESAJ; GMUD EPROC</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>23/03–03/04/26</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Worker CNJ; fila unificada; captura CNJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sprint 7</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06–17/04/26</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Webhook CNJ; fila 137k corrigida; desligamento parceiras (BUG-05..07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sprint 8</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>20/04–01/05/26</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Token compartilhado; fallback; tratamento de retornos (2 devs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Sprint 9</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>04–15/05/26</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Segredo de justiça por instância (escopo adicional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sprint 10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>18–29/05/26</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Validação E2E; retry webhook (BUG-08..09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sprint 11</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>01–12/06/26</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Em and.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Fase 6 — GMUD, deploy, 2ª instância (em andamento)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TOTAL / MÉDIA</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Disc.+11 sprints</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>147 (dev)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>~14</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Dev concluído 01/06/26 (+~30 dias). Fase 6 em andamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>RESULTADOS DE TESTES — SÍNTESE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Nível / Tipo</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Itens</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Defeitos</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Referência</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Testes de desempenho (EPROC)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>fluxo c/ múltiplos workers</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>REL-VV §2 (Fase 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Testes de integração (CNJ + webhook)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>fluxo completo</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>BUG-05..07 (corrigidos)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>REL-VV §2 (Fase 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Testes de fluxo / E2E</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>sucesso, fallback, erro parcial</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Aprovado por amostragem</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>REL-VV §2 (Fase 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Testes de persistência</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>movimentações por instância</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>REL-VV §2 (Fase 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Critérios de aceite</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CA01–CA07</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>7/7 validados</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>VV-AASPCNJ01-001 §3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -7058,8 +8983,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13" ht="21.75" customHeight="1" s="59">
       <c r="A13" s="62" t="inlineStr">
         <is>
@@ -7683,7 +9606,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="124" t="inlineStr">
         <is>
@@ -8134,7 +10056,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="21.75" customHeight="1" s="59">
       <c r="A16" s="62" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(GEST): corrige inversões de data (fim<início)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_CNJ/GEST-AASPCNJ01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_CNJ/GEST-AASPCNJ01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -2156,6 +2156,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="21.75" customHeight="1" s="59">
       <c r="A22" s="62" t="inlineStr">
         <is>
@@ -2649,6 +2650,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="21.75" customHeight="1" s="59">
       <c r="A12" s="62" t="inlineStr">
         <is>
@@ -2768,6 +2770,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="58" t="inlineStr">
         <is>
@@ -3071,6 +3074,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="58" t="inlineStr">
         <is>
@@ -4897,12 +4901,12 @@
       </c>
       <c r="C10" s="70" t="inlineStr">
         <is>
+          <t>09/02/2026</t>
+        </is>
+      </c>
+      <c r="D10" s="70" t="inlineStr">
+        <is>
           <t>14/02/2026</t>
-        </is>
-      </c>
-      <c r="D10" s="70" t="inlineStr">
-        <is>
-          <t>09/02/2026</t>
         </is>
       </c>
       <c r="E10" s="74" t="inlineStr">
@@ -7012,12 +7016,12 @@
       </c>
       <c r="C8" s="121" t="inlineStr">
         <is>
+          <t>09/02/2026</t>
+        </is>
+      </c>
+      <c r="D8" s="121" t="inlineStr">
+        <is>
           <t>14/02/2026</t>
-        </is>
-      </c>
-      <c r="D8" s="121" t="inlineStr">
-        <is>
-          <t>09/02/2026</t>
         </is>
       </c>
       <c r="E8" s="121" t="inlineStr">
@@ -8258,37 +8262,37 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="58" t="inlineStr">
         <is>
           <t>T-39</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="58" t="inlineStr">
         <is>
           <t>Hotfix de contenção (homologação): NullReference no consumidor da fila — v241</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="58" t="inlineStr">
         <is>
           <t>Jun/2026</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="58" t="inlineStr">
         <is>
           <t>Jun/2026</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="58" t="inlineStr">
         <is>
           <t>F6</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="58" t="inlineStr">
         <is>
           <t>RNF02</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G42" s="58" t="inlineStr">
         <is>
           <t>Concluída</t>
         </is>
@@ -9022,6 +9026,8 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13" ht="21.75" customHeight="1" s="59">
       <c r="A13" s="62" t="inlineStr">
         <is>
@@ -9645,6 +9651,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="124" t="inlineStr">
         <is>
@@ -10095,6 +10102,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="21.75" customHeight="1" s="59">
       <c r="A16" s="62" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(CNJ): migração Azure DevOps → GitLab + evidências e correções
- Plataforma/terminologia: Azure DevOps → GitLab; Pull Request → Merge Request
- Evidências GitLab alinhadas ao conteúdo real: branches, MR !12/!13 (DoD/aprovação),
  tags v2.0.0/v2.0.1/v2.0.2, pipeline #236, estrutura do repo (estrutura_cnj, .gitlab-ci.yml)
- Removidos prints do Azure (devops_cnj_*); estrutura_cnj substitui estrutura_WorkerAndamentos
- Planilha GEST: plataforma corrigida e ref de evidência EV-* → REL-VV-AASPCNJ01-001
- Headers: placeholder "Versão Data" preenchido (INDICE 1.5; CAP 1.1 + prefixo); docs alterados em v1.1
- Registros mantidos .docx-only (remoção das fontes .md)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_CNJ/GEST-AASPCNJ01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_CNJ/GEST-AASPCNJ01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -2061,7 +2061,7 @@
       </c>
       <c r="C17" s="74" t="inlineStr">
         <is>
-          <t>GCO — Azure DevOps</t>
+          <t>GCO — GitLab</t>
         </is>
       </c>
       <c r="D17" s="71" t="inlineStr">
@@ -9027,8 +9027,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13" ht="21.75" customHeight="1" s="59">
       <c r="A13" s="62" t="inlineStr">
         <is>
@@ -10093,7 +10091,7 @@
       </c>
       <c r="E14" s="74" t="inlineStr">
         <is>
-          <t>EV-AzureDevOps-CNJ-001 (Run #128)</t>
+          <t>REL-VV-AASPCNJ01-001</t>
         </is>
       </c>
       <c r="F14" s="74" t="inlineStr">

</xml_diff>

<commit_message>
auditoria geral (CNJ/AASPCNJ01): registros alinhados ao GitLab
- reconciliacao dos registros do projeto (GCO, ITP, REV, GEST) ao estado atual do instance aasp/cnj

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_CNJ/GEST-AASPCNJ01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_CNJ/GEST-AASPCNJ01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -2748,7 +2748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" style="59" min="1" max="1"/>
@@ -2768,6 +2768,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="58" t="inlineStr">
         <is>
@@ -3071,6 +3072,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="58" t="inlineStr">
         <is>
@@ -3856,14 +3858,51 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="58" t="inlineStr">
-        <is>
-          <t>TOTAL — 20 histórias</t>
-        </is>
-      </c>
-      <c r="D36" s="58" t="inlineStr">
-        <is>
-          <t>155</t>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>US-21</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Como time técnico, quero avaliar alternativa ao Puppeteer no crawler EPROC/ESAJ (reduzir bloqueio por firewall)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>RNF robustez</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>EP-07</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>🟡 Em and.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="58" t="inlineStr">
+        <is>
+          <t>TOTAL — 21 histórias</t>
+        </is>
+      </c>
+      <c r="D37" s="58" t="inlineStr">
+        <is>
+          <t>160</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" style="59" min="1" max="1"/>
@@ -3898,6 +3937,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="58" t="inlineStr">
         <is>
@@ -4452,117 +4492,133 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="58" t="inlineStr">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sprint 12</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>15–26/06/26</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Estudo de alternativa ao Puppeteer; GMUD/implantação</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="58" t="inlineStr">
         <is>
           <t>TOTAL / MÉDIA</t>
         </is>
       </c>
-      <c r="B18" s="58" t="inlineStr">
+      <c r="B19" s="58" t="inlineStr">
         <is>
           <t>Disc.+11 sprints</t>
         </is>
       </c>
-      <c r="C18" s="58" t="inlineStr">
+      <c r="C19" s="58" t="inlineStr">
         <is>
           <t>155</t>
         </is>
       </c>
-      <c r="D18" s="58" t="inlineStr">
+      <c r="D19" s="58" t="inlineStr">
         <is>
           <t>147 (dev)</t>
         </is>
       </c>
-      <c r="E18" s="58" t="inlineStr">
+      <c r="E19" s="58" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F18" s="58" t="inlineStr">
+      <c r="F19" s="58" t="inlineStr">
         <is>
           <t>~14</t>
         </is>
       </c>
-      <c r="G18" s="58" t="inlineStr">
+      <c r="G19" s="58" t="inlineStr">
         <is>
           <t>10 (9 dev + 1 contenção v241)</t>
         </is>
       </c>
-      <c r="H18" s="58" t="inlineStr">
+      <c r="H19" s="58" t="inlineStr">
         <is>
           <t>Dev concluído 01/06/26 (+~30 dias). Fase 6 em andamento.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="58" t="inlineStr">
-        <is>
-          <t>RESULTADOS DE TESTES — SÍNTESE</t>
-        </is>
-      </c>
-    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="58" t="inlineStr">
         <is>
-          <t>Nível / Tipo</t>
-        </is>
-      </c>
-      <c r="B21" s="58" t="inlineStr">
-        <is>
-          <t>Itens</t>
-        </is>
-      </c>
-      <c r="C21" s="58" t="inlineStr">
-        <is>
-          <t>Resultado</t>
-        </is>
-      </c>
-      <c r="D21" s="58" t="inlineStr">
-        <is>
-          <t>Defeitos</t>
-        </is>
-      </c>
-      <c r="H21" s="58" t="inlineStr">
-        <is>
-          <t>Referência</t>
+          <t>RESULTADOS DE TESTES — SÍNTESE</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="58" t="inlineStr">
         <is>
-          <t>Testes de desempenho (EPROC)</t>
+          <t>Nível / Tipo</t>
         </is>
       </c>
       <c r="B22" s="58" t="inlineStr">
         <is>
-          <t>fluxo c/ múltiplos workers</t>
+          <t>Itens</t>
         </is>
       </c>
       <c r="C22" s="58" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Resultado</t>
         </is>
       </c>
       <c r="D22" s="58" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Defeitos</t>
         </is>
       </c>
       <c r="H22" s="58" t="inlineStr">
         <is>
-          <t>REL-VV §2 (Fase 2)</t>
+          <t>Referência</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="58" t="inlineStr">
         <is>
-          <t>Testes de integração (CNJ + webhook)</t>
+          <t>Testes de desempenho (EPROC)</t>
         </is>
       </c>
       <c r="B23" s="58" t="inlineStr">
         <is>
-          <t>fluxo completo</t>
+          <t>fluxo c/ múltiplos workers</t>
         </is>
       </c>
       <c r="C23" s="58" t="inlineStr">
@@ -4572,56 +4628,56 @@
       </c>
       <c r="D23" s="58" t="inlineStr">
         <is>
-          <t>BUG-05..07 (corrigidos)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H23" s="58" t="inlineStr">
         <is>
-          <t>REL-VV §2 (Fase 4)</t>
+          <t>REL-VV §2 (Fase 2)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="58" t="inlineStr">
         <is>
-          <t>Testes de fluxo / E2E</t>
+          <t>Testes de integração (CNJ + webhook)</t>
         </is>
       </c>
       <c r="B24" s="58" t="inlineStr">
         <is>
-          <t>sucesso, fallback, erro parcial</t>
+          <t>fluxo completo</t>
         </is>
       </c>
       <c r="C24" s="58" t="inlineStr">
         <is>
-          <t>Aprovado por amostragem</t>
+          <t>Aprovado</t>
         </is>
       </c>
       <c r="D24" s="58" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>BUG-05..07 (corrigidos)</t>
         </is>
       </c>
       <c r="H24" s="58" t="inlineStr">
         <is>
-          <t>REL-VV §2 (Fase 5)</t>
+          <t>REL-VV §2 (Fase 4)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="58" t="inlineStr">
         <is>
-          <t>Testes de persistência</t>
+          <t>Testes de fluxo / E2E</t>
         </is>
       </c>
       <c r="B25" s="58" t="inlineStr">
         <is>
-          <t>movimentações por instância</t>
+          <t>sucesso, fallback, erro parcial</t>
         </is>
       </c>
       <c r="C25" s="58" t="inlineStr">
         <is>
-          <t>Aprovado</t>
+          <t>Aprovado por amostragem</t>
         </is>
       </c>
       <c r="D25" s="58" t="inlineStr">
@@ -4638,32 +4694,60 @@
     <row r="26">
       <c r="A26" s="58" t="inlineStr">
         <is>
+          <t>Testes de persistência</t>
+        </is>
+      </c>
+      <c r="B26" s="58" t="inlineStr">
+        <is>
+          <t>movimentações por instância</t>
+        </is>
+      </c>
+      <c r="C26" s="58" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="D26" s="58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H26" s="58" t="inlineStr">
+        <is>
+          <t>REL-VV §2 (Fase 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="58" t="inlineStr">
+        <is>
           <t>Critérios de aceite</t>
         </is>
       </c>
-      <c r="B26" s="58" t="inlineStr">
+      <c r="B27" s="58" t="inlineStr">
         <is>
           <t>CA01–CA07</t>
         </is>
       </c>
-      <c r="C26" s="58" t="inlineStr">
+      <c r="C27" s="58" t="inlineStr">
         <is>
           <t>7/7 validados</t>
         </is>
       </c>
-      <c r="D26" s="58" t="inlineStr">
+      <c r="D27" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H26" s="58" t="inlineStr">
+      <c r="H27" s="58" t="inlineStr">
         <is>
           <t>VV-AASPCNJ01-001 §3</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="58" t="inlineStr">
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="58" t="inlineStr">
         <is>
           <t>Nota: SP = esforço de desenvolvimento por sprint (modelagem retroativa); o merge em develop pode cair em sprint posterior ao desenvolvimento. Discovery + 11 sprints = 12 ciclos; 155 SP planejados.</t>
         </is>

</xml_diff>